<commit_message>
Update announcements — 2026-08-20T08:58:42.432Z
</commit_message>
<xml_diff>
--- a/Subject_Scheduler.xlsx
+++ b/Subject_Scheduler.xlsx
@@ -1634,7 +1634,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E4"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -1670,26 +1670,9 @@
         <v>Date</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>ann_1787216314068_o7ngbp</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Test</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Hi</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Bert</v>
-      </c>
-      <c r="E5" t="str">
-        <v>2026-08-20T08:58:34.068Z</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update schedule — 2026-08-20T08:59:24.551Z
</commit_message>
<xml_diff>
--- a/Subject_Scheduler.xlsx
+++ b/Subject_Scheduler.xlsx
@@ -401,6 +401,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L18"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" customWidth="1"/>
+    <col min="3" max="3" width="20.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+    <col min="6" max="6" width="11.83203125" customWidth="1"/>
+    <col min="7" max="7" width="18.83203125" customWidth="1"/>
+    <col min="8" max="8" width="30.83203125" customWidth="1"/>
+    <col min="9" max="9" width="22.83203125" customWidth="1"/>
+    <col min="10" max="10" width="12.83203125" customWidth="1"/>
+    <col min="11" max="11" width="16.83203125" customWidth="1"/>
+    <col min="12" max="12" width="24.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -472,8 +486,20 @@
       <c r="G5" t="str">
         <v>Mon: Online / Fri: Room 307</v>
       </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
       <c r="K5" t="str">
         <v>1st Sem</v>
+      </c>
+      <c r="L5" t="str">
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -498,8 +524,20 @@
       <c r="G6" t="str">
         <v>Mon: Online / Wed: Room 302</v>
       </c>
+      <c r="H6" t="str">
+        <v/>
+      </c>
+      <c r="I6" t="str">
+        <v/>
+      </c>
+      <c r="J6" t="str">
+        <v/>
+      </c>
       <c r="K6" t="str">
         <v>1st Sem</v>
+      </c>
+      <c r="L6" t="str">
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -527,8 +565,17 @@
       <c r="H7" t="str">
         <v>https://classroom.google.com/u/3/c/ODc0NzY4NDkwNTc0</v>
       </c>
+      <c r="I7" t="str">
+        <v/>
+      </c>
+      <c r="J7" t="str">
+        <v/>
+      </c>
       <c r="K7" t="str">
         <v>1st Sem</v>
+      </c>
+      <c r="L7" t="str">
+        <v/>
       </c>
     </row>
     <row r="8">
@@ -556,8 +603,17 @@
       <c r="H8" t="str">
         <v>https://classroom.google.com/c/ODU1ODc5MTczMjEx</v>
       </c>
+      <c r="I8" t="str">
+        <v/>
+      </c>
+      <c r="J8" t="str">
+        <v/>
+      </c>
       <c r="K8" t="str">
         <v>1st Sem</v>
+      </c>
+      <c r="L8" t="str">
+        <v/>
       </c>
     </row>
     <row r="9">
@@ -585,11 +641,17 @@
       <c r="H9" t="str">
         <v>https://classroom.google.com/c/ODU1ODgxNzY3NTQw?cjc=jl3v4fto</v>
       </c>
+      <c r="I9" t="str">
+        <v/>
+      </c>
       <c r="J9" t="str">
         <v>2026-2027</v>
       </c>
       <c r="K9" t="str">
         <v>1st Sem</v>
+      </c>
+      <c r="L9" t="str">
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -617,11 +679,17 @@
       <c r="H10" t="str">
         <v>https://classroom.google.com/c/ODU1ODgxNzY3NTQw?cjc=jl3v4fto</v>
       </c>
+      <c r="I10" t="str">
+        <v/>
+      </c>
       <c r="J10" t="str">
         <v>2026-2027</v>
       </c>
       <c r="K10" t="str">
         <v>1st Sem</v>
+      </c>
+      <c r="L10" t="str">
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -649,8 +717,17 @@
       <c r="H11" t="str">
         <v>https://classroom.google.com/c/ODU1ODc5MTczMjEx</v>
       </c>
+      <c r="I11" t="str">
+        <v/>
+      </c>
+      <c r="J11" t="str">
+        <v/>
+      </c>
       <c r="K11" t="str">
         <v>1st Sem</v>
+      </c>
+      <c r="L11" t="str">
+        <v/>
       </c>
     </row>
     <row r="12">
@@ -678,8 +755,17 @@
       <c r="H12" t="str">
         <v>https://classroom.google.com/u/3/c/ODc0NzY4NDkwNTc0</v>
       </c>
+      <c r="I12" t="str">
+        <v/>
+      </c>
+      <c r="J12" t="str">
+        <v/>
+      </c>
       <c r="K12" t="str">
         <v>1st Sem</v>
+      </c>
+      <c r="L12" t="str">
+        <v/>
       </c>
     </row>
     <row r="13">
@@ -704,8 +790,20 @@
       <c r="G13" t="str">
         <v>Mon: Online / Wed: Room 302</v>
       </c>
+      <c r="H13" t="str">
+        <v/>
+      </c>
+      <c r="I13" t="str">
+        <v/>
+      </c>
+      <c r="J13" t="str">
+        <v/>
+      </c>
       <c r="K13" t="str">
         <v>1st Sem</v>
+      </c>
+      <c r="L13" t="str">
+        <v/>
       </c>
     </row>
     <row r="14">
@@ -733,11 +831,17 @@
       <c r="H14" t="str">
         <v>https://classroom.google.com/c/ODc0NzQ1NDA2MDEw</v>
       </c>
+      <c r="I14" t="str">
+        <v>https://meet.google.com/landing?authuser=0</v>
+      </c>
       <c r="J14" t="str">
         <v>2026-2027</v>
       </c>
       <c r="K14" t="str">
         <v>1st Sem</v>
+      </c>
+      <c r="L14" t="str">
+        <v/>
       </c>
     </row>
     <row r="15">
@@ -765,11 +869,17 @@
       <c r="H15" t="str">
         <v>https://classroom.google.com/c/ODc0NzQ1NDA2MDEw</v>
       </c>
+      <c r="I15" t="str">
+        <v/>
+      </c>
       <c r="J15" t="str">
         <v>2026-2027</v>
       </c>
       <c r="K15" t="str">
         <v>1st Sem</v>
+      </c>
+      <c r="L15" t="str">
+        <v/>
       </c>
     </row>
     <row r="16">
@@ -794,8 +904,20 @@
       <c r="G16" t="str">
         <v>Mon: Online / Fri: 307</v>
       </c>
+      <c r="H16" t="str">
+        <v/>
+      </c>
+      <c r="I16" t="str">
+        <v/>
+      </c>
+      <c r="J16" t="str">
+        <v/>
+      </c>
       <c r="K16" t="str">
         <v>1st Sem</v>
+      </c>
+      <c r="L16" t="str">
+        <v/>
       </c>
     </row>
     <row r="17">
@@ -823,11 +945,17 @@
       <c r="H17" t="str">
         <v>https://classroom.google.com/c/ODU1ODc5OTMyNDEz</v>
       </c>
+      <c r="I17" t="str">
+        <v/>
+      </c>
       <c r="J17" t="str">
         <v>2026-2027</v>
       </c>
       <c r="K17" t="str">
         <v>1st Sem</v>
+      </c>
+      <c r="L17" t="str">
+        <v/>
       </c>
     </row>
     <row r="18">
@@ -855,15 +983,20 @@
       <c r="H18" t="str">
         <v>https://classroom.google.com/c/ODU1ODc5NzkxODc0</v>
       </c>
+      <c r="I18" t="str">
+        <v/>
+      </c>
       <c r="J18" t="str">
         <v>2026-2027</v>
       </c>
       <c r="K18" t="str">
         <v>1st Sem</v>
       </c>
+      <c r="L18" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:L18"/>
   </ignoredErrors>
@@ -1635,13 +1768,6 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E4"/>
-  <cols>
-    <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="30.83203125" customWidth="1"/>
-    <col min="3" max="3" width="60.83203125" customWidth="1"/>
-    <col min="4" max="4" width="22.83203125" customWidth="1"/>
-    <col min="5" max="5" width="22.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">

</xml_diff>

<commit_message>
Update announcements — 2026-08-20T09:13:00.354Z
</commit_message>
<xml_diff>
--- a/Subject_Scheduler.xlsx
+++ b/Subject_Scheduler.xlsx
@@ -401,20 +401,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L18"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="24.83203125" customWidth="1"/>
-    <col min="3" max="3" width="20.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" customWidth="1"/>
-    <col min="6" max="6" width="11.83203125" customWidth="1"/>
-    <col min="7" max="7" width="18.83203125" customWidth="1"/>
-    <col min="8" max="8" width="30.83203125" customWidth="1"/>
-    <col min="9" max="9" width="22.83203125" customWidth="1"/>
-    <col min="10" max="10" width="12.83203125" customWidth="1"/>
-    <col min="11" max="11" width="16.83203125" customWidth="1"/>
-    <col min="12" max="12" width="24.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1767,7 +1753,14 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
+  <cols>
+    <col min="1" max="1" width="16.83203125" customWidth="1"/>
+    <col min="2" max="2" width="30.83203125" customWidth="1"/>
+    <col min="3" max="3" width="60.83203125" customWidth="1"/>
+    <col min="4" max="4" width="22.83203125" customWidth="1"/>
+    <col min="5" max="5" width="22.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1796,9 +1789,37 @@
         <v>Date</v>
       </c>
     </row>
+    <row r="5" xml:space="preserve">
+      <c r="A5" t="str">
+        <v>ann_1787217180347_3r0q7r</v>
+      </c>
+      <c r="B5" t="str">
+        <v>IMPORTANT ANNOUNCEMENT!!!</v>
+      </c>
+      <c r="C5" t="str" xml:space="preserve">
+        <v xml:space="preserve">Subject: System Analysis and Design
+Topic: Group Research Project
+Group composition: 1-3
+Deadline of submission of group members: August 22, 2026 - 5:00PM PHT
+Requirements and Guidelines:
+- 5 Research Title per member (5 x No. of member)
+- Allowed:
+1. Web-Based or Application Systems (Desktop/Mobile)
+- Prohibited:
+1. More than 3 members
+2. A.I.-generated shits
+3. Walang bitaw na  member</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Bert</v>
+      </c>
+      <c r="E5" t="str">
+        <v>2026-08-20T09:13:00.347Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update schedule — 2026-08-20T10:25:14.637Z
</commit_message>
<xml_diff>
--- a/Subject_Scheduler.xlsx
+++ b/Subject_Scheduler.xlsx
@@ -401,6 +401,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L18"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" customWidth="1"/>
+    <col min="3" max="3" width="20.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+    <col min="6" max="6" width="11.83203125" customWidth="1"/>
+    <col min="7" max="7" width="18.83203125" customWidth="1"/>
+    <col min="8" max="8" width="30.83203125" customWidth="1"/>
+    <col min="9" max="9" width="22.83203125" customWidth="1"/>
+    <col min="10" max="10" width="12.83203125" customWidth="1"/>
+    <col min="11" max="11" width="16.83203125" customWidth="1"/>
+    <col min="12" max="12" width="24.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -472,8 +486,20 @@
       <c r="G5" t="str">
         <v>Mon: Online / Fri: Room 307</v>
       </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
       <c r="K5" t="str">
         <v>1st Sem</v>
+      </c>
+      <c r="L5" t="str">
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -498,8 +524,20 @@
       <c r="G6" t="str">
         <v>Mon: Online / Wed: Room 302</v>
       </c>
+      <c r="H6" t="str">
+        <v/>
+      </c>
+      <c r="I6" t="str">
+        <v/>
+      </c>
+      <c r="J6" t="str">
+        <v/>
+      </c>
       <c r="K6" t="str">
         <v>1st Sem</v>
+      </c>
+      <c r="L6" t="str">
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -530,8 +568,14 @@
       <c r="I7" t="str">
         <v>https://meet.google.com/oav-esck-wpt?authuser=0</v>
       </c>
+      <c r="J7" t="str">
+        <v/>
+      </c>
       <c r="K7" t="str">
         <v>1st Sem</v>
+      </c>
+      <c r="L7" t="str">
+        <v/>
       </c>
     </row>
     <row r="8">
@@ -562,8 +606,14 @@
       <c r="I8" t="str">
         <v>https://meet.google.com/yjs-eqov-wpm?authuser=0</v>
       </c>
+      <c r="J8" t="str">
+        <v/>
+      </c>
       <c r="K8" t="str">
         <v>1st Sem</v>
+      </c>
+      <c r="L8" t="str">
+        <v/>
       </c>
     </row>
     <row r="9">
@@ -600,6 +650,9 @@
       <c r="K9" t="str">
         <v>1st Sem</v>
       </c>
+      <c r="L9" t="str">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -635,6 +688,9 @@
       <c r="K10" t="str">
         <v>1st Sem</v>
       </c>
+      <c r="L10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -664,8 +720,14 @@
       <c r="I11" t="str">
         <v>https://meet.google.com/yjs-eqov-wpm?authuser=0</v>
       </c>
+      <c r="J11" t="str">
+        <v/>
+      </c>
       <c r="K11" t="str">
         <v>1st Sem</v>
+      </c>
+      <c r="L11" t="str">
+        <v/>
       </c>
     </row>
     <row r="12">
@@ -696,8 +758,14 @@
       <c r="I12" t="str">
         <v>https://meet.google.com/oav-esck-wpt?authuser=0</v>
       </c>
+      <c r="J12" t="str">
+        <v/>
+      </c>
       <c r="K12" t="str">
         <v>1st Sem</v>
+      </c>
+      <c r="L12" t="str">
+        <v/>
       </c>
     </row>
     <row r="13">
@@ -722,8 +790,20 @@
       <c r="G13" t="str">
         <v>Mon: Online / Wed: Room 302</v>
       </c>
+      <c r="H13" t="str">
+        <v/>
+      </c>
+      <c r="I13" t="str">
+        <v/>
+      </c>
+      <c r="J13" t="str">
+        <v/>
+      </c>
       <c r="K13" t="str">
         <v>1st Sem</v>
+      </c>
+      <c r="L13" t="str">
+        <v/>
       </c>
     </row>
     <row r="14">
@@ -760,6 +840,9 @@
       <c r="K14" t="str">
         <v>1st Sem</v>
       </c>
+      <c r="L14" t="str">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -795,6 +878,9 @@
       <c r="K15" t="str">
         <v>1st Sem</v>
       </c>
+      <c r="L15" t="str">
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -818,8 +904,20 @@
       <c r="G16" t="str">
         <v>Mon: Online / Fri: 307</v>
       </c>
+      <c r="H16" t="str">
+        <v/>
+      </c>
+      <c r="I16" t="str">
+        <v/>
+      </c>
+      <c r="J16" t="str">
+        <v/>
+      </c>
       <c r="K16" t="str">
         <v>1st Sem</v>
+      </c>
+      <c r="L16" t="str">
+        <v/>
       </c>
     </row>
     <row r="17">
@@ -847,11 +945,17 @@
       <c r="H17" t="str">
         <v>https://classroom.google.com/c/ODU1ODc5OTMyNDEz</v>
       </c>
+      <c r="I17" t="str">
+        <v/>
+      </c>
       <c r="J17" t="str">
         <v>2026-2027</v>
       </c>
       <c r="K17" t="str">
         <v>1st Sem</v>
+      </c>
+      <c r="L17" t="str">
+        <v/>
       </c>
     </row>
     <row r="18">
@@ -879,15 +983,20 @@
       <c r="H18" t="str">
         <v>https://classroom.google.com/c/ODU1ODc5NzkxODc0</v>
       </c>
+      <c r="I18" t="str">
+        <v/>
+      </c>
       <c r="J18" t="str">
         <v>2026-2027</v>
       </c>
       <c r="K18" t="str">
         <v>1st Sem</v>
       </c>
+      <c r="L18" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:L18"/>
   </ignoredErrors>
@@ -1800,16 +1909,6 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H5"/>
-  <cols>
-    <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="30.83203125" customWidth="1"/>
-    <col min="3" max="3" width="60.83203125" customWidth="1"/>
-    <col min="4" max="4" width="22.83203125" customWidth="1"/>
-    <col min="5" max="5" width="22.83203125" customWidth="1"/>
-    <col min="6" max="6" width="22.83203125" customWidth="1"/>
-    <col min="7" max="7" width="22.83203125" customWidth="1"/>
-    <col min="8" max="8" width="8.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">

</xml_diff>

<commit_message>
Update announcements — 2026-08-20T10:47:13.942Z
</commit_message>
<xml_diff>
--- a/Subject_Scheduler.xlsx
+++ b/Subject_Scheduler.xlsx
@@ -401,20 +401,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L18"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="24.83203125" customWidth="1"/>
-    <col min="3" max="3" width="20.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" customWidth="1"/>
-    <col min="6" max="6" width="11.83203125" customWidth="1"/>
-    <col min="7" max="7" width="18.83203125" customWidth="1"/>
-    <col min="8" max="8" width="30.83203125" customWidth="1"/>
-    <col min="9" max="9" width="22.83203125" customWidth="1"/>
-    <col min="10" max="10" width="12.83203125" customWidth="1"/>
-    <col min="11" max="11" width="16.83203125" customWidth="1"/>
-    <col min="12" max="12" width="24.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1908,7 +1894,17 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
+  <cols>
+    <col min="1" max="1" width="16.83203125" customWidth="1"/>
+    <col min="2" max="2" width="30.83203125" customWidth="1"/>
+    <col min="3" max="3" width="60.83203125" customWidth="1"/>
+    <col min="4" max="4" width="22.83203125" customWidth="1"/>
+    <col min="5" max="5" width="22.83203125" customWidth="1"/>
+    <col min="6" max="6" width="22.83203125" customWidth="1"/>
+    <col min="7" max="7" width="22.83203125" customWidth="1"/>
+    <col min="8" max="8" width="8.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1983,9 +1979,36 @@
         <v>1</v>
       </c>
     </row>
+    <row r="6" xml:space="preserve">
+      <c r="A6" t="str">
+        <v>ann_1787222833867_b89eet</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Holiday Tomorrow: NINOY AQUINO DAY</v>
+      </c>
+      <c r="C6" t="str" xml:space="preserve">
+        <v xml:space="preserve">To learn more about this, watch here:
+https://youtu.be/dQw4w9WgXcQ?si=q1vhwdXlbSRL9W-H</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Jerome</v>
+      </c>
+      <c r="E6" t="str">
+        <v>2026-08-20T10:47:13.867Z</v>
+      </c>
+      <c r="F6" t="str">
+        <v>2026-08-20T10:47:13.867Z</v>
+      </c>
+      <c r="G6" t="str">
+        <v>2026-08-20T15:59:59.000Z</v>
+      </c>
+      <c r="H6" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update announcements — 2026-08-20T11:27:29.632Z
</commit_message>
<xml_diff>
--- a/Subject_Scheduler.xlsx
+++ b/Subject_Scheduler.xlsx
@@ -1964,13 +1964,13 @@
 3. Walang bitaw na  member</v>
       </c>
       <c r="D5" t="str">
-        <v>JC_</v>
+        <v>Bert</v>
       </c>
       <c r="E5" t="str">
         <v>2026-08-20T09:13:00.347Z</v>
       </c>
       <c r="F5" t="str">
-        <v>2026-08-20T10:19:17.322Z</v>
+        <v>2026-08-20T11:27:29.612Z</v>
       </c>
       <c r="G5" t="str">
         <v>2026-08-22T15:59:59.000Z</v>

</xml_diff>

<commit_message>
Update announcements — 2026-08-20T17:09:33.694Z
</commit_message>
<xml_diff>
--- a/Subject_Scheduler.xlsx
+++ b/Subject_Scheduler.xlsx
@@ -1991,16 +1991,16 @@
 https://youtu.be/dQw4w9WgXcQ?si=q1vhwdXlbSRL9W-H</v>
       </c>
       <c r="D6" t="str">
-        <v>Jerome</v>
+        <v>Bert</v>
       </c>
       <c r="E6" t="str">
         <v>2026-08-20T10:47:13.867Z</v>
       </c>
       <c r="F6" t="str">
-        <v>2026-08-20T10:47:13.867Z</v>
+        <v>2026-08-20T17:09:33.670Z</v>
       </c>
       <c r="G6" t="str">
-        <v>2026-08-20T15:59:59.000Z</v>
+        <v>2026-08-21T15:59:59.000Z</v>
       </c>
       <c r="H6" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Update announcements — 2026-08-20T17:10:18.654Z
</commit_message>
<xml_diff>
--- a/Subject_Scheduler.xlsx
+++ b/Subject_Scheduler.xlsx
@@ -1984,7 +1984,7 @@
         <v>ann_1787222833867_b89eet</v>
       </c>
       <c r="B6" t="str">
-        <v>Holiday Tomorrow: NINOY AQUINO DAY</v>
+        <v>Holiday: August 21, 2026 PH - NINOY AQUINO DAY</v>
       </c>
       <c r="C6" t="str" xml:space="preserve">
         <v xml:space="preserve">To learn more about this, watch here:
@@ -1997,7 +1997,7 @@
         <v>2026-08-20T10:47:13.867Z</v>
       </c>
       <c r="F6" t="str">
-        <v>2026-08-20T17:09:33.670Z</v>
+        <v>2026-08-20T17:10:18.646Z</v>
       </c>
       <c r="G6" t="str">
         <v>2026-08-21T15:59:59.000Z</v>

</xml_diff>

<commit_message>
Update announcements — 2026-08-20T17:10:56.262Z
</commit_message>
<xml_diff>
--- a/Subject_Scheduler.xlsx
+++ b/Subject_Scheduler.xlsx
@@ -1947,7 +1947,7 @@
         <v>ann_1787217180347_3r0q7r</v>
       </c>
       <c r="B5" t="str">
-        <v>IMPORTANT ANNOUNCEMENT!!!</v>
+        <v>Update: System Analysis and Design</v>
       </c>
       <c r="C5" t="str" xml:space="preserve">
         <v xml:space="preserve">Subject: System Analysis and Design
@@ -1970,7 +1970,7 @@
         <v>2026-08-20T09:13:00.347Z</v>
       </c>
       <c r="F5" t="str">
-        <v>2026-08-20T11:27:29.612Z</v>
+        <v>2026-08-20T17:10:56.251Z</v>
       </c>
       <c r="G5" t="str">
         <v>2026-08-22T15:59:59.000Z</v>

</xml_diff>

<commit_message>
Update announcements — 2026-08-21T17:21:22.653Z
</commit_message>
<xml_diff>
--- a/Subject_Scheduler.xlsx
+++ b/Subject_Scheduler.xlsx
@@ -1894,7 +1894,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H5"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -1979,36 +1979,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" xml:space="preserve">
-      <c r="A6" t="str">
-        <v>ann_1787222833867_b89eet</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Holiday: August 21, 2026 PH - NINOY AQUINO DAY</v>
-      </c>
-      <c r="C6" t="str" xml:space="preserve">
-        <v xml:space="preserve">To learn more about this, watch here:
-https://youtu.be/dQw4w9WgXcQ?si=q1vhwdXlbSRL9W-H</v>
-      </c>
-      <c r="D6" t="str">
-        <v>Bert</v>
-      </c>
-      <c r="E6" t="str">
-        <v>2026-08-20T10:47:13.867Z</v>
-      </c>
-      <c r="F6" t="str">
-        <v>2026-08-20T17:10:18.646Z</v>
-      </c>
-      <c r="G6" t="str">
-        <v>2026-08-21T15:59:59.000Z</v>
-      </c>
-      <c r="H6" t="b">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Flashcards: Add Flashcard — 2026-08-22T17:49:45.733Z
</commit_message>
<xml_diff>
--- a/Subject_Scheduler.xlsx
+++ b/Subject_Scheduler.xlsx
@@ -7,6 +7,8 @@
     <sheet name="Legend" sheetId="2" r:id="rId2"/>
     <sheet name="Valid_Users" sheetId="3" r:id="rId3"/>
     <sheet name="Announcements" sheetId="4" r:id="rId4"/>
+    <sheet name="Flashcards" sheetId="5" r:id="rId5"/>
+    <sheet name="Audit_Log" sheetId="6" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
@@ -1895,16 +1897,6 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H5"/>
-  <cols>
-    <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="30.83203125" customWidth="1"/>
-    <col min="3" max="3" width="60.83203125" customWidth="1"/>
-    <col min="4" max="4" width="22.83203125" customWidth="1"/>
-    <col min="5" max="5" width="22.83203125" customWidth="1"/>
-    <col min="6" max="6" width="22.83203125" customWidth="1"/>
-    <col min="7" max="7" width="22.83203125" customWidth="1"/>
-    <col min="8" max="8" width="8.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1984,4 +1976,166 @@
     <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H5"/>
+  <cols>
+    <col min="1" max="1" width="16.83203125" customWidth="1"/>
+    <col min="2" max="2" width="26.83203125" customWidth="1"/>
+    <col min="3" max="3" width="10.83203125" customWidth="1"/>
+    <col min="4" max="4" width="40.83203125" customWidth="1"/>
+    <col min="5" max="5" width="40.83203125" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+    <col min="7" max="7" width="20.83203125" customWidth="1"/>
+    <col min="8" max="8" width="20.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Flashcards — Personalized School Record Management System</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Master accounts add/edit/delete cards here; anyone signed in can review them.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>ID</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Deck</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Type</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Front</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Back</v>
+      </c>
+      <c r="F4" t="str">
+        <v>CreatedBy</v>
+      </c>
+      <c r="G4" t="str">
+        <v>CreatedAt</v>
+      </c>
+      <c r="H4" t="str">
+        <v>UpdatedAt</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>card_1787420985723_5bswth</v>
+      </c>
+      <c r="B5" t="str">
+        <v>DM101-Plannin</v>
+      </c>
+      <c r="C5" t="str">
+        <v>basic</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Front Test</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Back Test</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Bert</v>
+      </c>
+      <c r="G5" t="str">
+        <v>2026-08-22T17:49:45.723Z</v>
+      </c>
+      <c r="H5" t="str">
+        <v>2026-08-22T17:49:45.723Z</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E6"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="20.83203125" customWidth="1"/>
+    <col min="3" max="3" width="10.83203125" customWidth="1"/>
+    <col min="4" max="4" width="20.83203125" customWidth="1"/>
+    <col min="5" max="5" width="42.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Audit Log — Personalized School Record Management System</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Read-only history of sign-ins and changes. Visible to Master accounts only, and not editable through any app UI.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Timestamp</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Actor</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Role</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Action</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Details</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>2026-08-23T01:48:01+08:00</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Bert</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Master</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Login</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Master</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>2026-08-23T01:49:45+08:00</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Bert</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Master</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Add Flashcard</v>
+      </c>
+      <c r="E6" t="str">
+        <v>DM101-Plannin</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E6"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Flashcards: Add Flashcard — 2026-08-22T17:50:39.981Z
</commit_message>
<xml_diff>
--- a/Subject_Scheduler.xlsx
+++ b/Subject_Scheduler.xlsx
@@ -1980,7 +1980,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -2054,16 +2054,42 @@
         <v>2026-08-22T17:49:45.723Z</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>card_1787421039976_2qwhp5</v>
+      </c>
+      <c r="B6" t="str">
+        <v>DM101-Planning</v>
+      </c>
+      <c r="C6" t="str">
+        <v>cloze</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Hello there _____.</v>
+      </c>
+      <c r="E6" t="str">
+        <v>My friend</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Bert</v>
+      </c>
+      <c r="G6" t="str">
+        <v>2026-08-22T17:50:39.976Z</v>
+      </c>
+      <c r="H6" t="str">
+        <v>2026-08-22T17:50:39.976Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H6"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -2133,9 +2159,26 @@
         <v>DM101-Plannin</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>2026-08-23T01:50:39+08:00</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Bert</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Master</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Add Flashcard</v>
+      </c>
+      <c r="E7" t="str">
+        <v>DM101-Planning — cloze</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Flashcards: Delete Flashcard — 2026-08-22T17:51:46.731Z
</commit_message>
<xml_diff>
--- a/Subject_Scheduler.xlsx
+++ b/Subject_Scheduler.xlsx
@@ -1980,7 +1980,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H5"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -2030,66 +2030,40 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>card_1787420985723_5bswth</v>
+        <v>card_1787421039976_2qwhp5</v>
       </c>
       <c r="B5" t="str">
-        <v>DM101-Plannin</v>
+        <v>DM101-Planning</v>
       </c>
       <c r="C5" t="str">
-        <v>basic</v>
+        <v>cloze</v>
       </c>
       <c r="D5" t="str">
-        <v>Front Test</v>
+        <v>Hello there _____.</v>
       </c>
       <c r="E5" t="str">
-        <v>Back Test</v>
+        <v>My friend</v>
       </c>
       <c r="F5" t="str">
         <v>Bert</v>
       </c>
       <c r="G5" t="str">
-        <v>2026-08-22T17:49:45.723Z</v>
+        <v>2026-08-22T17:50:39.976Z</v>
       </c>
       <c r="H5" t="str">
-        <v>2026-08-22T17:49:45.723Z</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>card_1787421039976_2qwhp5</v>
-      </c>
-      <c r="B6" t="str">
-        <v>DM101-Planning</v>
-      </c>
-      <c r="C6" t="str">
-        <v>cloze</v>
-      </c>
-      <c r="D6" t="str">
-        <v>Hello there _____.</v>
-      </c>
-      <c r="E6" t="str">
-        <v>My friend</v>
-      </c>
-      <c r="F6" t="str">
-        <v>Bert</v>
-      </c>
-      <c r="G6" t="str">
-        <v>2026-08-22T17:50:39.976Z</v>
-      </c>
-      <c r="H6" t="str">
         <v>2026-08-22T17:50:39.976Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E9"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -2176,9 +2150,43 @@
         <v>DM101-Planning — cloze</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>2026-08-23T01:51:12+08:00</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Bert</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Master</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Login</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Master</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>2026-08-23T01:51:46+08:00</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Bert</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Master</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Delete Flashcard</v>
+      </c>
+      <c r="E9" t="str">
+        <v>DM101-Plannin — Front Test</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Flashcards: Delete Flashcard — 2026-08-22T17:52:41.367Z
</commit_message>
<xml_diff>
--- a/Subject_Scheduler.xlsx
+++ b/Subject_Scheduler.xlsx
@@ -1980,7 +1980,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H4"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -2028,42 +2028,16 @@
         <v>UpdatedAt</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>card_1787421039976_2qwhp5</v>
-      </c>
-      <c r="B5" t="str">
-        <v>DM101-Planning</v>
-      </c>
-      <c r="C5" t="str">
-        <v>cloze</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Hello there _____.</v>
-      </c>
-      <c r="E5" t="str">
-        <v>My friend</v>
-      </c>
-      <c r="F5" t="str">
-        <v>Bert</v>
-      </c>
-      <c r="G5" t="str">
-        <v>2026-08-22T17:50:39.976Z</v>
-      </c>
-      <c r="H5" t="str">
-        <v>2026-08-22T17:50:39.976Z</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E11"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -2184,9 +2158,43 @@
         <v>DM101-Plannin — Front Test</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>2026-08-23T01:52:26+08:00</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Bert</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Master</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Login</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Master</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>2026-08-23T01:52:41+08:00</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Bert</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Master</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Delete Flashcard</v>
+      </c>
+      <c r="E11" t="str">
+        <v>DM101-Planning — Hello there _____.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update announcements — 2026-08-22T17:53:21.893Z
</commit_message>
<xml_diff>
--- a/Subject_Scheduler.xlsx
+++ b/Subject_Scheduler.xlsx
@@ -1896,7 +1896,17 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H4"/>
+  <cols>
+    <col min="1" max="1" width="16.83203125" customWidth="1"/>
+    <col min="2" max="2" width="30.83203125" customWidth="1"/>
+    <col min="3" max="3" width="60.83203125" customWidth="1"/>
+    <col min="4" max="4" width="22.83203125" customWidth="1"/>
+    <col min="5" max="5" width="22.83203125" customWidth="1"/>
+    <col min="6" max="6" width="22.83203125" customWidth="1"/>
+    <col min="7" max="7" width="22.83203125" customWidth="1"/>
+    <col min="8" max="8" width="8.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1934,46 +1944,9 @@
         <v>Pinned</v>
       </c>
     </row>
-    <row r="5" xml:space="preserve">
-      <c r="A5" t="str">
-        <v>ann_1787217180347_3r0q7r</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Update: System Analysis and Design</v>
-      </c>
-      <c r="C5" t="str" xml:space="preserve">
-        <v xml:space="preserve">Subject: System Analysis and Design
-Topic: Group Research Project
-Group composition: 1-3
-Deadline of submission of group members: August 22, 2026 - 5:00PM PHT
-Requirements and Guidelines:
-- 5 Research Title per member (5 x No. of member)
-- Allowed:
-1. Web-Based or Application Systems (Desktop/Mobile)
-- Prohibited:
-1. More than 3 members
-2. A.I.-generated shits
-3. Walang bitaw na  member</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Bert</v>
-      </c>
-      <c r="E5" t="str">
-        <v>2026-08-20T09:13:00.347Z</v>
-      </c>
-      <c r="F5" t="str">
-        <v>2026-08-20T17:10:56.251Z</v>
-      </c>
-      <c r="G5" t="str">
-        <v>2026-08-22T15:59:59.000Z</v>
-      </c>
-      <c r="H5" t="b">
-        <v>1</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H4"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1981,16 +1954,6 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H4"/>
-  <cols>
-    <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="26.83203125" customWidth="1"/>
-    <col min="3" max="3" width="10.83203125" customWidth="1"/>
-    <col min="4" max="4" width="40.83203125" customWidth="1"/>
-    <col min="5" max="5" width="40.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-    <col min="7" max="7" width="20.83203125" customWidth="1"/>
-    <col min="8" max="8" width="20.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2037,7 +2000,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E13"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -2192,9 +2155,43 @@
         <v>DM101-Planning — Hello there _____.</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>2026-08-23T01:53:16+08:00</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Bert</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Master</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Login</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Master</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>2026-08-23T01:53:21+08:00</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Bert</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Master</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Delete Announcement</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Update: System Analysis and Design</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update announcements — 2026-08-22T17:59:08.734Z
</commit_message>
<xml_diff>
--- a/Subject_Scheduler.xlsx
+++ b/Subject_Scheduler.xlsx
@@ -1896,7 +1896,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H5"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -1944,9 +1944,35 @@
         <v>Pinned</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>ann_1787421548723_uui0z2</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Reminder</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Drink water daily ❤️</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Bert</v>
+      </c>
+      <c r="E5" t="str">
+        <v>2026-08-22T17:59:08.723Z</v>
+      </c>
+      <c r="F5" t="str">
+        <v>2026-08-22T17:59:08.723Z</v>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2000,7 +2026,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E15"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -2189,9 +2215,43 @@
         <v>Update: System Analysis and Design</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>2026-08-23T01:56:26+08:00</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Bert</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Master</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Login</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Master</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>2026-08-23T01:59:08+08:00</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Bert</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Master</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Add Announcement</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Reminder</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E15"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update schedule — by test_dummy
</commit_message>
<xml_diff>
--- a/Subject_Scheduler.xlsx
+++ b/Subject_Scheduler.xlsx
@@ -490,7 +490,7 @@
         <v>Mon: Online / Fri: Room 307</v>
       </c>
       <c r="H5" t="str">
-        <v/>
+        <v>https://classroom.google.com/c/ODc0NzI1NDEzMjYw/m/ODc1NTY5NDgxOTMy/details</v>
       </c>
       <c r="I5" t="str">
         <v>https://meet.google.com/uue-itbf-scf</v>
@@ -4879,7 +4879,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E187"/>
+  <dimension ref="A1:E188"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -8026,9 +8026,26 @@
         <v>MAT110 — Quantitative Methods</v>
       </c>
     </row>
+    <row r="188">
+      <c r="A188" t="str">
+        <v>2026-09-05T20:06:34+08:00</v>
+      </c>
+      <c r="B188" t="str">
+        <v>test_dummy</v>
+      </c>
+      <c r="C188" t="str">
+        <v>Master</v>
+      </c>
+      <c r="D188" t="str">
+        <v>Edit Subject</v>
+      </c>
+      <c r="E188" t="str">
+        <v>DM103 — Business Process Design and Management</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E187"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E188"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Flashcards: Add Flashcard — by Bert
</commit_message>
<xml_diff>
--- a/Subject_Scheduler.xlsx
+++ b/Subject_Scheduler.xlsx
@@ -404,20 +404,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L18"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="24.83203125" customWidth="1"/>
-    <col min="3" max="3" width="20.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" customWidth="1"/>
-    <col min="6" max="6" width="11.83203125" customWidth="1"/>
-    <col min="7" max="7" width="18.83203125" customWidth="1"/>
-    <col min="8" max="8" width="30.83203125" customWidth="1"/>
-    <col min="9" max="9" width="22.83203125" customWidth="1"/>
-    <col min="10" max="10" width="12.83203125" customWidth="1"/>
-    <col min="11" max="11" width="16.83203125" customWidth="1"/>
-    <col min="12" max="12" width="24.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2153,7 +2139,17 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H107"/>
+  <dimension ref="A1:H108"/>
+  <cols>
+    <col min="1" max="1" width="16.83203125" customWidth="1"/>
+    <col min="2" max="2" width="26.83203125" customWidth="1"/>
+    <col min="3" max="3" width="10.83203125" customWidth="1"/>
+    <col min="4" max="4" width="40.83203125" customWidth="1"/>
+    <col min="5" max="5" width="40.83203125" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+    <col min="7" max="7" width="20.83203125" customWidth="1"/>
+    <col min="8" max="8" width="20.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4869,17 +4865,43 @@
         <v>2026-08-29T18:15:52.396Z</v>
       </c>
     </row>
+    <row r="108" xml:space="preserve">
+      <c r="A108" t="str">
+        <v>card_1788688176189_x0znxp</v>
+      </c>
+      <c r="B108" t="str">
+        <v>MAT110 - Lesson1</v>
+      </c>
+      <c r="C108" t="str">
+        <v>cloze</v>
+      </c>
+      <c r="D108" t="str" xml:space="preserve">
+        <v xml:space="preserve">_____ is a systematic record of facts, such as numbers, words, measurements, observations or just
+descriptions of things from which conclusions may be drawn.</v>
+      </c>
+      <c r="E108" t="str">
+        <v>Data</v>
+      </c>
+      <c r="F108" t="str">
+        <v>Bert</v>
+      </c>
+      <c r="G108" t="str">
+        <v>2026-09-06T09:49:36.189Z</v>
+      </c>
+      <c r="H108" t="str">
+        <v>2026-09-06T09:49:36.189Z</v>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H107"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H108"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E193"/>
+  <dimension ref="A1:E196"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -8128,9 +8150,60 @@
         <v>MAT110 — Quantitative Methods</v>
       </c>
     </row>
+    <row r="194">
+      <c r="A194" t="str">
+        <v>2026-09-06T17:46:40+08:00</v>
+      </c>
+      <c r="B194" t="str">
+        <v>Bert</v>
+      </c>
+      <c r="C194" t="str">
+        <v>Master</v>
+      </c>
+      <c r="D194" t="str">
+        <v>Login</v>
+      </c>
+      <c r="E194" t="str">
+        <v>Master</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="str">
+        <v>2026-09-06T17:46:51+08:00</v>
+      </c>
+      <c r="B195" t="str">
+        <v>Bert</v>
+      </c>
+      <c r="C195" t="str">
+        <v>Master</v>
+      </c>
+      <c r="D195" t="str">
+        <v>Login</v>
+      </c>
+      <c r="E195" t="str">
+        <v>Master</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="str">
+        <v>2026-09-06T17:49:36+08:00</v>
+      </c>
+      <c r="B196" t="str">
+        <v>Bert</v>
+      </c>
+      <c r="C196" t="str">
+        <v>Master</v>
+      </c>
+      <c r="D196" t="str">
+        <v>Add Flashcard</v>
+      </c>
+      <c r="E196" t="str">
+        <v>MAT110 - Lesson1 — cloze</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E193"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E196"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Flashcards: Edit Flashcard — by Bert
</commit_message>
<xml_diff>
--- a/Subject_Scheduler.xlsx
+++ b/Subject_Scheduler.xlsx
@@ -4865,7 +4865,7 @@
         <v>2026-08-29T18:15:52.396Z</v>
       </c>
     </row>
-    <row r="108" xml:space="preserve">
+    <row r="108">
       <c r="A108" t="str">
         <v>card_1788688176189_x0znxp</v>
       </c>
@@ -4875,9 +4875,8 @@
       <c r="C108" t="str">
         <v>cloze</v>
       </c>
-      <c r="D108" t="str" xml:space="preserve">
-        <v xml:space="preserve">_____ is a systematic record of facts, such as numbers, words, measurements, observations or just
-descriptions of things from which conclusions may be drawn.</v>
+      <c r="D108" t="str">
+        <v>_____ is a systematic record of facts, such as numbers, words, measurements, observations or just descriptions of things from which conclusions may be drawn.</v>
       </c>
       <c r="E108" t="str">
         <v>Data</v>
@@ -4889,7 +4888,7 @@
         <v>2026-09-06T09:49:36.189Z</v>
       </c>
       <c r="H108" t="str">
-        <v>2026-09-06T09:49:36.189Z</v>
+        <v>2026-09-06T09:49:53.083Z</v>
       </c>
     </row>
   </sheetData>
@@ -4901,7 +4900,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E196"/>
+  <dimension ref="A1:E197"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -8201,9 +8200,26 @@
         <v>MAT110 - Lesson1 — cloze</v>
       </c>
     </row>
+    <row r="197">
+      <c r="A197" t="str">
+        <v>2026-09-06T17:49:53+08:00</v>
+      </c>
+      <c r="B197" t="str">
+        <v>Bert</v>
+      </c>
+      <c r="C197" t="str">
+        <v>Master</v>
+      </c>
+      <c r="D197" t="str">
+        <v>Edit Flashcard</v>
+      </c>
+      <c r="E197" t="str">
+        <v>MAT110 - Lesson1 — cloze</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E196"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E197"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>